<commit_message>
Update Dakdekker BE variants: new ReviewDescription template with AantalJaren
</commit_message>
<xml_diff>
--- a/branch_files/Dakdekker/Eigen merk/BE/variants.xlsx
+++ b/branch_files/Dakdekker/Eigen merk/BE/variants.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\menno\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB44D84C-526C-4361-A3BF-E3393364DE95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FABFF951-02BE-4668-86C3-B21C9BA0C618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="85">
   <si>
     <t>Vlaamse dakcampagnes Eigen Merk – korte en lange plaatsvarianten</t>
   </si>
@@ -182,9 +182,6 @@
     <t>Met Jarenlange Ervaring</t>
   </si>
   <si>
-    <t>https://peeters-dakwerken.be/</t>
-  </si>
-  <si>
     <t>Toegepaste logica en Vlaamse positionering</t>
   </si>
   <si>
@@ -254,12 +251,6 @@
     <t>Reviewfallback</t>
   </si>
   <si>
-    <t>Geen reviewclaim</t>
-  </si>
-  <si>
-    <t>Peeters benadrukt gediplomeerde dakwerkers, ervaren stielmannen, garantie, kwaliteit en 24/24 bereikbaarheid.</t>
-  </si>
-  <si>
     <t>Primaire keuze</t>
   </si>
   <si>
@@ -275,10 +266,16 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Indien geen reviews aanwezig</t>
-  </si>
-  <si>
-    <t>Peeters benadrukt gediplomeerde dakwerkers, [ReviewDescription], garantie, kwaliteit en 24/24 bereikbaarheid.</t>
+    <t>[AantalJaren] jaar garantie, ervaren stielmannen en 24 op 24 bereikbaar bij dringende dakproblemen.</t>
+  </si>
+  <si>
+    <t>[AantalJaren] jaar garantie, [ReviewDescription] en 24 op 24 bereikbaar bij dringende dakproblemen.</t>
+  </si>
+  <si>
+    <t>Indien aantal sterren ingevuld wordt het '5 sterren' in plaats van [ReviewDescription], indien geen cijfer ingevuld wordt het lange variant.</t>
+  </si>
+  <si>
+    <t>Indien cijfer aanwezig bij aantal sterren 'Beoordeeld met 5 sterren' Indien geen reviews aanwezig wordt het lange variant.</t>
   </si>
 </sst>
 </file>
@@ -355,7 +352,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -369,12 +366,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -603,26 +603,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="20.85" customHeight="1">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
     </row>
     <row r="2" spans="1:7" ht="27.15" customHeight="1">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
     </row>
     <row r="4" spans="1:7" ht="27.15" customHeight="1">
       <c r="A4" s="2" t="s">
@@ -967,9 +967,9 @@
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="27.6">
-      <c r="A19" s="7" t="s">
-        <v>82</v>
+    <row r="19" spans="1:7" ht="69">
+      <c r="A19" s="5" t="s">
+        <v>79</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>51</v>
@@ -980,25 +980,25 @@
       <c r="D19" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="E19" s="8" t="s">
+      <c r="E19" s="6" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="41.4">
-      <c r="A20" s="7" t="s">
+    <row r="20" spans="1:7" ht="69">
+      <c r="A20" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B20" t="s">
+        <v>82</v>
+      </c>
+      <c r="C20" t="s">
+        <v>82</v>
+      </c>
+      <c r="D20" t="s">
+        <v>81</v>
+      </c>
+      <c r="E20" s="9" t="s">
         <v>83</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="E20" s="8" t="s">
-        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1012,7 +1012,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -1022,67 +1022,67 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="17.399999999999999">
-      <c r="A1" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
+      <c r="A1" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="27.6">
       <c r="A4" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="27.6">
       <c r="A5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>65</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -1090,13 +1090,13 @@
         <v>24</v>
       </c>
       <c r="B7" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -1104,41 +1104,27 @@
         <v>25</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C8" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="27.6">
       <c r="A9" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="27.6">
-      <c r="A10" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix Description 3 [AantalJaren] unreplaced: detect 'geen cijfer' as no_review rule, apply eigen placeholders in city branch
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/branch_files/Dakdekker/Eigen merk/BE/variants.xlsx
+++ b/branch_files/Dakdekker/Eigen merk/BE/variants.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\menno\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FABFF951-02BE-4668-86C3-B21C9BA0C618}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7E89F9C-F797-40A3-A642-35F276937D41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -269,13 +269,13 @@
     <t>[AantalJaren] jaar garantie, ervaren stielmannen en 24 op 24 bereikbaar bij dringende dakproblemen.</t>
   </si>
   <si>
-    <t>[AantalJaren] jaar garantie, [ReviewDescription] en 24 op 24 bereikbaar bij dringende dakproblemen.</t>
-  </si>
-  <si>
     <t>Indien aantal sterren ingevuld wordt het '5 sterren' in plaats van [ReviewDescription], indien geen cijfer ingevuld wordt het lange variant.</t>
   </si>
   <si>
     <t>Indien cijfer aanwezig bij aantal sterren 'Beoordeeld met 5 sterren' Indien geen reviews aanwezig wordt het lange variant.</t>
+  </si>
+  <si>
+    <t>[AantalJaren] Jaar Garantie, [ReviewDescription] en 24 op 24 bereikbaar bij dringende dakproblemen.</t>
   </si>
 </sst>
 </file>
@@ -352,7 +352,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -375,9 +375,6 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -596,7 +593,8 @@
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="4" width="52" customWidth="1"/>
+    <col min="2" max="2" width="90.8984375" customWidth="1"/>
+    <col min="3" max="4" width="52" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
     <col min="6" max="6" width="16" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
@@ -981,7 +979,7 @@
         <v>52</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="69">
@@ -989,16 +987,16 @@
         <v>80</v>
       </c>
       <c r="B20" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C20" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D20" t="s">
         <v>81</v>
       </c>
-      <c r="E20" s="9" t="s">
-        <v>83</v>
+      <c r="E20" s="6" t="s">
+        <v>82</v>
       </c>
     </row>
   </sheetData>

</xml_diff>